<commit_message>
feat: atualizei o calendário.
</commit_message>
<xml_diff>
--- a/courseware/calendario.xlsx
+++ b/courseware/calendario.xlsx
@@ -98,13 +98,13 @@
     <t>Numpy.</t>
   </si>
   <si>
-    <t>Usar Numpy para representar vetores e suas</t>
+    <t>Usar Numpy para representar vetores e suas operações</t>
   </si>
   <si>
     <t>vetores/numpy01.ipynb</t>
   </si>
   <si>
-    <t>Numpy como ferramenta para visualizar</t>
+    <t>Numpy como ferramenta.</t>
   </si>
   <si>
     <t>Aplicar Numpy e álgebra vetorial para simular uma situação-problema.</t>
@@ -122,7 +122,7 @@
     <t>vetores/projecoes.ipynb</t>
   </si>
   <si>
-    <t>Embeddings</t>
+    <t>Embeddings.</t>
   </si>
   <si>
     <t>Aplicar Numpy para visualizar espaços de embeddings e suas propriedades.</t>
@@ -158,7 +158,7 @@
     <t>matrizes/inversa.md</t>
   </si>
   <si>
-    <t>Determinantes</t>
+    <t>Determinantes.</t>
   </si>
   <si>
     <t>Determinar se um sistema linear tem solução ou não.</t>
@@ -167,7 +167,7 @@
     <t>matrizes/determinante.md</t>
   </si>
   <si>
-    <t>Transformações afins</t>
+    <t>Transformações afins.</t>
   </si>
   <si>
     <t>Relacionar sistemas lineares com transformações geométricas.</t>

</xml_diff>